<commit_message>
Unify client templates and add Yandex auth
</commit_message>
<xml_diff>
--- a/templates/detmir_upload_template.xlsx
+++ b/templates/detmir_upload_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Детский Мир" sheetId="1" r:id="R2ff1ac098abe48a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как загружать" sheetId="2" r:id="R837c9156cc2d405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Детский Мир" sheetId="1" r:id="R234edf307d1f4e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как использовать" sheetId="2" r:id="Re64a333514b74236"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,6 +17,11 @@
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="334155"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -36,11 +41,6 @@
       <x:color rgb="FFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="334155"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
   <x:fills count="6">
     <x:fill>
@@ -48,6 +48,11 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="F8FAFC"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -64,11 +69,6 @@
         <x:fgColor rgb="DBEAFE"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="F8FAFC"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="4">
     <x:border/>
@@ -83,54 +83,67 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -289,101 +302,166 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="33.56999969482422" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="27.860000610351562" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30.709999084472656" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22.139999389648438" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="107.86000061035156" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="12" t="str">
+      <x:c r="A1" s="8" t="str">
+        <x:v>Артикул UpdatPic. Нужен, если фото уже спарсены и лежат в локальном каталоге сервиса.</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>Штрихкод товара. Если штрихкодов несколько, указывайте целевой код для выгрузки этой строки.</x:v>
+      </x:c>
+      <x:c r="C1" s="8" t="str">
+        <x:v>Источник фото: каталог или ссылки. Если не заполнено, сервис выберет ссылки при наличии URL, иначе каталог.</x:v>
+      </x:c>
+      <x:c r="D1" s="8" t="str">
+        <x:v>Прямая ссылка на изображение, можно вставить несколько. Поддерживаются прямые URL и публичные ссылки из раздела Файлы Яндекс Диска. Разделители: перевод строки, пробел, запятая или ;</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="22" t="str">
         <x:v>article</x:v>
       </x:c>
-      <x:c r="B1" s="12" t="str">
-        <x:v>Штрихкод товара</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="13" t="str">
+      <x:c r="B2" s="22" t="str">
+        <x:v>Штрихкод товара*</x:v>
+      </x:c>
+      <x:c r="C2" s="22" t="str">
+        <x:v>Источник фото</x:v>
+      </x:c>
+      <x:c r="D2" s="22" t="str">
+        <x:v>Ссылки на изображения товара</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="20" t="str">
         <x:v>TSR-10025</x:v>
       </x:c>
-      <x:c r="B2" s="13" t="str">
-        <x:v>4607000012345</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="13" t="str">
-        <x:v>TSR-10026</x:v>
-      </x:c>
-      <x:c r="B3" s="13" t="str">
-        <x:v>4607000012346</x:v>
-      </x:c>
+      <x:c r="B3" s="20" t="str">
+        <x:v>4660120067909</x:v>
+      </x:c>
+      <x:c r="C3" s="20" t="str">
+        <x:v>каталог</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="14" t="str"/>
+      <x:c r="A4" s="20" t="str"/>
+      <x:c r="B4" s="20" t="str">
+        <x:v>4660120067916</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str">
+        <x:v>ссылки</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="str">
+        <x:v>https://static.detmir.st/media_out/523/698/3698523/1500/0.jpg
+https://static.detmir.st/media_out/523/698/3698523/1500/1.jpg</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="14"/>
-      <x:c r="B5" s="14"/>
+      <x:c r="A5" s="20" t="str"/>
+      <x:c r="B5" s="20" t="str">
+        <x:v>4660120067923</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="str">
+        <x:v>ссылки</x:v>
+      </x:c>
+      <x:c r="D5" s="20" t="str">
+        <x:v>https://disk.yandex.ru/d/example-public-link</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="14"/>
-      <x:c r="B6" s="14"/>
+      <x:c r="A6" s="23" t="str"/>
+      <x:c r="B6" s="23" t="str"/>
+      <x:c r="C6" s="23" t="str"/>
+      <x:c r="D6" s="23" t="str"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="14"/>
-      <x:c r="B7" s="14"/>
+      <x:c r="A7" s="23"/>
+      <x:c r="B7" s="23"/>
+      <x:c r="C7" s="23"/>
+      <x:c r="D7" s="23"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="14"/>
-      <x:c r="B8" s="14"/>
+      <x:c r="A8" s="23"/>
+      <x:c r="B8" s="23"/>
+      <x:c r="C8" s="23"/>
+      <x:c r="D8" s="23"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="14"/>
-      <x:c r="B9" s="14"/>
+      <x:c r="A9" s="23"/>
+      <x:c r="B9" s="23"/>
+      <x:c r="C9" s="23"/>
+      <x:c r="D9" s="23"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="14"/>
-      <x:c r="B10" s="14"/>
+      <x:c r="A10" s="23"/>
+      <x:c r="B10" s="23"/>
+      <x:c r="C10" s="23"/>
+      <x:c r="D10" s="23"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="14"/>
-      <x:c r="B11" s="14"/>
+      <x:c r="A11" s="23"/>
+      <x:c r="B11" s="23"/>
+      <x:c r="C11" s="23"/>
+      <x:c r="D11" s="23"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="14"/>
-      <x:c r="B12" s="14"/>
+      <x:c r="A12" s="23"/>
+      <x:c r="B12" s="23"/>
+      <x:c r="C12" s="23"/>
+      <x:c r="D12" s="23"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="14"/>
-      <x:c r="B13" s="14"/>
+      <x:c r="A13" s="23"/>
+      <x:c r="B13" s="23"/>
+      <x:c r="C13" s="23"/>
+      <x:c r="D13" s="23"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="14"/>
-      <x:c r="B14" s="14"/>
+      <x:c r="A14" s="23"/>
+      <x:c r="B14" s="23"/>
+      <x:c r="C14" s="23"/>
+      <x:c r="D14" s="23"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="14"/>
-      <x:c r="B15" s="14"/>
+      <x:c r="A15" s="23"/>
+      <x:c r="B15" s="23"/>
+      <x:c r="C15" s="23"/>
+      <x:c r="D15" s="23"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="14"/>
-      <x:c r="B16" s="14"/>
+      <x:c r="A16" s="23"/>
+      <x:c r="B16" s="23"/>
+      <x:c r="C16" s="23"/>
+      <x:c r="D16" s="23"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="14"/>
-      <x:c r="B17" s="14"/>
+      <x:c r="A17" s="23"/>
+      <x:c r="B17" s="23"/>
+      <x:c r="C17" s="23"/>
+      <x:c r="D17" s="23"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="14"/>
-      <x:c r="B18" s="14"/>
+      <x:c r="A18" s="23"/>
+      <x:c r="B18" s="23"/>
+      <x:c r="C18" s="23"/>
+      <x:c r="D18" s="23"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="14"/>
+      <x:c r="A19" s="23"/>
+      <x:c r="B19" s="23"/>
+      <x:c r="C19" s="23"/>
+      <x:c r="D19" s="23"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="14"/>
+      <x:c r="A20" s="23"/>
+      <x:c r="B20" s="23"/>
+      <x:c r="C20" s="23"/>
+      <x:c r="D20" s="23"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -394,110 +472,120 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.140000343322754" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="50.709999084472656" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="45" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22.139999389648438" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="55" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46.43000030517578" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="12" t="str">
-        <x:v>Шаблон для Детского Мира</x:v>
-      </x:c>
-      <x:c r="B1" s="12"/>
-      <x:c r="C1" s="12"/>
+      <x:c r="A1" s="22" t="str">
+        <x:v>Шаблон Детский Мир</x:v>
+      </x:c>
+      <x:c r="B1" s="22"/>
+      <x:c r="C1" s="22"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="14"/>
-      <x:c r="B2" s="14"/>
-      <x:c r="C2" s="14"/>
+      <x:c r="A2" s="23"/>
+      <x:c r="B2" s="23"/>
+      <x:c r="C2" s="23"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="30" t="str">
-        <x:v>Пункт</x:v>
-      </x:c>
-      <x:c r="B3" s="30" t="str">
-        <x:v>Что делать</x:v>
-      </x:c>
-      <x:c r="C3" s="30" t="str">
-        <x:v>Комментарий</x:v>
+      <x:c r="A3" s="32" t="str">
+        <x:v>Сценарий</x:v>
+      </x:c>
+      <x:c r="B3" s="32" t="str">
+        <x:v>Что заполнить</x:v>
+      </x:c>
+      <x:c r="C3" s="32" t="str">
+        <x:v>Что получите</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="28" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B4" s="28" t="str">
-        <x:v>На листе Детский Мир заполнить article и Штрихкод товара</x:v>
-      </x:c>
-      <x:c r="C4" s="28" t="str">
-        <x:v>Каждая строка = один товар в UpdatPic</x:v>
+      <x:c r="A4" s="8" t="str">
+        <x:v>А. Фото уже спарсены</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>article + Штрихкод товара. Ссылки оставить пустыми или написать Источник фото = каталог</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>ZIP с файлами Штрихкод_01, Штрихкод_02 и т.д.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="28" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B5" s="28" t="str">
-        <x:v>Загрузить этот файл в раздел Клиенты и выбрать клиента Детский Мир</x:v>
-      </x:c>
-      <x:c r="C5" s="28" t="str">
-        <x:v>Сервис упакует фото в ZIP</x:v>
+      <x:c r="A5" s="8" t="str">
+        <x:v>Б. Готовые ссылки уже есть</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>Штрихкод товара + Ссылки на изображения товара. article можно не заполнять и указать Источник фото = ссылки</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>Excel со ссылками для загрузки в Детский Мир</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="28" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B6" s="28" t="str">
-        <x:v>После сборки архива имена файлов будут вида Штрихкод_01, Штрихкод_02 и т.д.</x:v>
-      </x:c>
-      <x:c r="C6" s="28" t="str">
-        <x:v>Пример: 4607000012345_01.jpg</x:v>
+      <x:c r="A6" s="8" t="str">
+        <x:v>Разделители</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>Перевод строки, пробел, запятая или ;</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="str">
+        <x:v>Сервис сам нормализует список</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="28" t="str">
-        <x:v>Формат</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="str">
-        <x:v>Допустимые файлы: jpg, jpeg, png, webp</x:v>
-      </x:c>
-      <x:c r="C7" s="28" t="str">
-        <x:v>UpdatPic сохранит подходящее расширение</x:v>
+      <x:c r="A7" s="8" t="str">
+        <x:v>Ограничение</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>Максимум 30 ссылок на товар</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>Лишние будут отброшены с предупреждением</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="28" t="str">
-        <x:v>Размер</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="str">
-        <x:v>Длинная сторона 1000-8000 px, до 1 МБ</x:v>
-      </x:c>
-      <x:c r="C8" s="28" t="str">
-        <x:v>Сервис уменьшит слишком большие изображения</x:v>
+      <x:c r="A8" s="8" t="str">
+        <x:v>Требования</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>Формат jpg/png/webp, длинная сторона 1000-8000 px, объём до 1 МБ</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>Для удалённых ссылок размеры и вес нужно проверять на стороне источника</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="28" t="str">
+      <x:c r="A9" s="8" t="str">
         <x:v>Важно</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
-        <x:v>Штрихкод товара даёт менеджер</x:v>
-      </x:c>
-      <x:c r="C9" s="28" t="str">
-        <x:v>Без него файлы нельзя правильно назвать для Детского Мира</x:v>
+      <x:c r="B9" s="8" t="str">
+        <x:v>Один и тот же файл можно смешивать: часть строк из каталога, часть по готовым ссылкам</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>Сервис отдаст оба результата, если нужны оба</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="28" t="str">
-        <x:v>Важно</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="str">
-        <x:v>Фото не должны быть перегружены, с водяными знаками, QR и посторонними логотипами</x:v>
-      </x:c>
-      <x:c r="C10" s="28" t="str">
-        <x:v>Это уже правило модерации клиента</x:v>
-      </x:c>
+      <x:c r="A10" s="8" t="str">
+        <x:v>Пример имени</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>4660120067909_01.jpg</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>Формат финального файла для локального каталога</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="8"/>
+      <x:c r="B11" s="8"/>
+      <x:c r="C11" s="8"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="8"/>
+      <x:c r="B12" s="8"/>
+      <x:c r="C12" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>